<commit_message>
Finalize secure checkout, payments, and email notifications
</commit_message>
<xml_diff>
--- a/server/seed/Product_Database.xlsx
+++ b/server/seed/Product_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://maelectricals.sharepoint.com/sites/ProjectCoordination/Shared Documents/MAE/Website/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="135" documentId="8_{EBC7D351-0979-4006-A801-EAB119450C32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C23EAFB1-679D-48C1-8D1A-B0F2E741DDF9}"/>
+  <xr:revisionPtr revIDLastSave="138" documentId="8_{EBC7D351-0979-4006-A801-EAB119450C32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6FF4B0C-894F-4161-8DA2-1567ED888C5E}"/>
   <bookViews>
-    <workbookView xWindow="1872" yWindow="5436" windowWidth="17280" windowHeight="8880" xr2:uid="{21F85595-19D1-4714-85EF-8F93F70DCA98}"/>
+    <workbookView xWindow="684" yWindow="828" windowWidth="17280" windowHeight="8880" xr2:uid="{21F85595-19D1-4714-85EF-8F93F70DCA98}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2893,6 +2893,9 @@
       <c r="E3" t="s">
         <v>32</v>
       </c>
+      <c r="G3">
+        <v>100</v>
+      </c>
       <c r="H3" t="s">
         <v>567</v>
       </c>
@@ -2925,6 +2928,9 @@
       <c r="E4" t="s">
         <v>31</v>
       </c>
+      <c r="G4">
+        <v>100</v>
+      </c>
       <c r="H4" t="s">
         <v>567</v>
       </c>
@@ -2956,6 +2962,9 @@
       </c>
       <c r="E5" t="s">
         <v>30</v>
+      </c>
+      <c r="G5">
+        <v>100</v>
       </c>
       <c r="H5" t="s">
         <v>567</v>
@@ -9137,7 +9146,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9797926-4691-4A32-A7E1-8BC3F4183B15}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9797926-4691-4A32-A7E1-8BC3F4183B15}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5032d0b3-1e0e-4943-a888-fd7360781fc5"/>
+    <ds:schemaRef ds:uri="d10c95b8-36b2-487f-b11e-2c8a90c74a0d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>